<commit_message>
Pre-fill Product Design 팀원 13명 명단
이요한(Yohan, 리더), 정수현, 문지선, 윤소현, 한수민, 이선진,
이재구, 조수경, 방채영, 윤세린, 심희정, 백신혜, 안유진

균등분배 시 1인당 약 284,563원 (3,699,320 ÷ 13).
사용내역 샘플 이름도 실제 팀원으로 교체.

https://claude.ai/code/session_01EJxm1Q1JyTJVR1M5kUU4Nw
</commit_message>
<xml_diff>
--- a/product_design_ttb_budget.xlsx
+++ b/product_design_ttb_budget.xlsx
@@ -1753,7 +1753,7 @@
     <row r="5">
       <c r="A5" s="16" t="inlineStr">
         <is>
-          <t>김디자이너</t>
+          <t>이요한(Yohan)</t>
         </is>
       </c>
       <c r="B5" s="9">
@@ -1765,12 +1765,16 @@
         <f>IF(A5="","",IF(ISNUMBER(C5),C5,B5))</f>
         <v/>
       </c>
-      <c r="E5" s="16" t="n"/>
+      <c r="E5" s="16" t="inlineStr">
+        <is>
+          <t>리더</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="16" t="inlineStr">
         <is>
-          <t>박디자이너</t>
+          <t>정수현(Gongdee)</t>
         </is>
       </c>
       <c r="B6" s="9">
@@ -1782,12 +1786,12 @@
         <f>IF(A6="","",IF(ISNUMBER(C6),C6,B6))</f>
         <v/>
       </c>
-      <c r="E6" s="16" t="n"/>
+      <c r="E6" s="16" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="16" t="inlineStr">
         <is>
-          <t>이디자이너</t>
+          <t>문지선(Sun)</t>
         </is>
       </c>
       <c r="B7" s="9">
@@ -1799,12 +1803,12 @@
         <f>IF(A7="","",IF(ISNUMBER(C7),C7,B7))</f>
         <v/>
       </c>
-      <c r="E7" s="16" t="n"/>
+      <c r="E7" s="16" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="16" t="inlineStr">
         <is>
-          <t>최디자이너</t>
+          <t>윤소현(Jenna)</t>
         </is>
       </c>
       <c r="B8" s="9">
@@ -1816,12 +1820,12 @@
         <f>IF(A8="","",IF(ISNUMBER(C8),C8,B8))</f>
         <v/>
       </c>
-      <c r="E8" s="16" t="n"/>
+      <c r="E8" s="16" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="16" t="inlineStr">
         <is>
-          <t>정디자이너</t>
+          <t>한수민(Stella)</t>
         </is>
       </c>
       <c r="B9" s="9">
@@ -1833,10 +1837,14 @@
         <f>IF(A9="","",IF(ISNUMBER(C9),C9,B9))</f>
         <v/>
       </c>
-      <c r="E9" s="16" t="n"/>
+      <c r="E9" s="16" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="16" t="inlineStr"/>
+      <c r="A10" s="16" t="inlineStr">
+        <is>
+          <t>이선진(Deeer)</t>
+        </is>
+      </c>
       <c r="B10" s="9">
         <f>IF(A10="","",총예산/COUNTA($A$5:$A$34))</f>
         <v/>
@@ -1846,10 +1854,14 @@
         <f>IF(A10="","",IF(ISNUMBER(C10),C10,B10))</f>
         <v/>
       </c>
-      <c r="E10" s="16" t="n"/>
+      <c r="E10" s="16" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="16" t="inlineStr"/>
+      <c r="A11" s="16" t="inlineStr">
+        <is>
+          <t>이재구(Jack)</t>
+        </is>
+      </c>
       <c r="B11" s="9">
         <f>IF(A11="","",총예산/COUNTA($A$5:$A$34))</f>
         <v/>
@@ -1859,10 +1871,14 @@
         <f>IF(A11="","",IF(ISNUMBER(C11),C11,B11))</f>
         <v/>
       </c>
-      <c r="E11" s="16" t="n"/>
+      <c r="E11" s="16" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="16" t="inlineStr"/>
+      <c r="A12" s="16" t="inlineStr">
+        <is>
+          <t>조수경(Skamie)</t>
+        </is>
+      </c>
       <c r="B12" s="9">
         <f>IF(A12="","",총예산/COUNTA($A$5:$A$34))</f>
         <v/>
@@ -1872,10 +1888,14 @@
         <f>IF(A12="","",IF(ISNUMBER(C12),C12,B12))</f>
         <v/>
       </c>
-      <c r="E12" s="16" t="n"/>
+      <c r="E12" s="16" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="16" t="inlineStr"/>
+      <c r="A13" s="16" t="inlineStr">
+        <is>
+          <t>방채영(Dana)</t>
+        </is>
+      </c>
       <c r="B13" s="9">
         <f>IF(A13="","",총예산/COUNTA($A$5:$A$34))</f>
         <v/>
@@ -1885,10 +1905,14 @@
         <f>IF(A13="","",IF(ISNUMBER(C13),C13,B13))</f>
         <v/>
       </c>
-      <c r="E13" s="16" t="n"/>
+      <c r="E13" s="16" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="16" t="inlineStr"/>
+      <c r="A14" s="16" t="inlineStr">
+        <is>
+          <t>윤세린(Selah)</t>
+        </is>
+      </c>
       <c r="B14" s="9">
         <f>IF(A14="","",총예산/COUNTA($A$5:$A$34))</f>
         <v/>
@@ -1898,10 +1922,14 @@
         <f>IF(A14="","",IF(ISNUMBER(C14),C14,B14))</f>
         <v/>
       </c>
-      <c r="E14" s="16" t="n"/>
+      <c r="E14" s="16" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="16" t="inlineStr"/>
+      <c r="A15" s="16" t="inlineStr">
+        <is>
+          <t>심희정(Lana)</t>
+        </is>
+      </c>
       <c r="B15" s="9">
         <f>IF(A15="","",총예산/COUNTA($A$5:$A$34))</f>
         <v/>
@@ -1911,10 +1939,14 @@
         <f>IF(A15="","",IF(ISNUMBER(C15),C15,B15))</f>
         <v/>
       </c>
-      <c r="E15" s="16" t="n"/>
+      <c r="E15" s="16" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="16" t="inlineStr"/>
+      <c r="A16" s="16" t="inlineStr">
+        <is>
+          <t>백신혜(Gina)</t>
+        </is>
+      </c>
       <c r="B16" s="9">
         <f>IF(A16="","",총예산/COUNTA($A$5:$A$34))</f>
         <v/>
@@ -1924,10 +1956,14 @@
         <f>IF(A16="","",IF(ISNUMBER(C16),C16,B16))</f>
         <v/>
       </c>
-      <c r="E16" s="16" t="n"/>
+      <c r="E16" s="16" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="16" t="inlineStr"/>
+      <c r="A17" s="16" t="inlineStr">
+        <is>
+          <t>안유진(Jinny)</t>
+        </is>
+      </c>
       <c r="B17" s="9">
         <f>IF(A17="","",총예산/COUNTA($A$5:$A$34))</f>
         <v/>
@@ -1937,7 +1973,7 @@
         <f>IF(A17="","",IF(ISNUMBER(C17),C17,B17))</f>
         <v/>
       </c>
-      <c r="E17" s="16" t="n"/>
+      <c r="E17" s="16" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="16" t="inlineStr"/>
@@ -1950,7 +1986,7 @@
         <f>IF(A18="","",IF(ISNUMBER(C18),C18,B18))</f>
         <v/>
       </c>
-      <c r="E18" s="16" t="n"/>
+      <c r="E18" s="16" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="16" t="inlineStr"/>
@@ -1963,7 +1999,7 @@
         <f>IF(A19="","",IF(ISNUMBER(C19),C19,B19))</f>
         <v/>
       </c>
-      <c r="E19" s="16" t="n"/>
+      <c r="E19" s="16" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="16" t="inlineStr"/>
@@ -1976,7 +2012,7 @@
         <f>IF(A20="","",IF(ISNUMBER(C20),C20,B20))</f>
         <v/>
       </c>
-      <c r="E20" s="16" t="n"/>
+      <c r="E20" s="16" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="16" t="inlineStr"/>
@@ -1989,7 +2025,7 @@
         <f>IF(A21="","",IF(ISNUMBER(C21),C21,B21))</f>
         <v/>
       </c>
-      <c r="E21" s="16" t="n"/>
+      <c r="E21" s="16" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="16" t="inlineStr"/>
@@ -2002,7 +2038,7 @@
         <f>IF(A22="","",IF(ISNUMBER(C22),C22,B22))</f>
         <v/>
       </c>
-      <c r="E22" s="16" t="n"/>
+      <c r="E22" s="16" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="16" t="inlineStr"/>
@@ -2015,7 +2051,7 @@
         <f>IF(A23="","",IF(ISNUMBER(C23),C23,B23))</f>
         <v/>
       </c>
-      <c r="E23" s="16" t="n"/>
+      <c r="E23" s="16" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="16" t="inlineStr"/>
@@ -2028,7 +2064,7 @@
         <f>IF(A24="","",IF(ISNUMBER(C24),C24,B24))</f>
         <v/>
       </c>
-      <c r="E24" s="16" t="n"/>
+      <c r="E24" s="16" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="16" t="inlineStr"/>
@@ -2041,7 +2077,7 @@
         <f>IF(A25="","",IF(ISNUMBER(C25),C25,B25))</f>
         <v/>
       </c>
-      <c r="E25" s="16" t="n"/>
+      <c r="E25" s="16" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="16" t="inlineStr"/>
@@ -2054,7 +2090,7 @@
         <f>IF(A26="","",IF(ISNUMBER(C26),C26,B26))</f>
         <v/>
       </c>
-      <c r="E26" s="16" t="n"/>
+      <c r="E26" s="16" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="16" t="inlineStr"/>
@@ -2067,7 +2103,7 @@
         <f>IF(A27="","",IF(ISNUMBER(C27),C27,B27))</f>
         <v/>
       </c>
-      <c r="E27" s="16" t="n"/>
+      <c r="E27" s="16" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="16" t="inlineStr"/>
@@ -2080,7 +2116,7 @@
         <f>IF(A28="","",IF(ISNUMBER(C28),C28,B28))</f>
         <v/>
       </c>
-      <c r="E28" s="16" t="n"/>
+      <c r="E28" s="16" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="16" t="inlineStr"/>
@@ -2093,7 +2129,7 @@
         <f>IF(A29="","",IF(ISNUMBER(C29),C29,B29))</f>
         <v/>
       </c>
-      <c r="E29" s="16" t="n"/>
+      <c r="E29" s="16" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="16" t="inlineStr"/>
@@ -2106,7 +2142,7 @@
         <f>IF(A30="","",IF(ISNUMBER(C30),C30,B30))</f>
         <v/>
       </c>
-      <c r="E30" s="16" t="n"/>
+      <c r="E30" s="16" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="16" t="inlineStr"/>
@@ -2119,7 +2155,7 @@
         <f>IF(A31="","",IF(ISNUMBER(C31),C31,B31))</f>
         <v/>
       </c>
-      <c r="E31" s="16" t="n"/>
+      <c r="E31" s="16" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="16" t="inlineStr"/>
@@ -2132,7 +2168,7 @@
         <f>IF(A32="","",IF(ISNUMBER(C32),C32,B32))</f>
         <v/>
       </c>
-      <c r="E32" s="16" t="n"/>
+      <c r="E32" s="16" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="16" t="inlineStr"/>
@@ -2145,7 +2181,7 @@
         <f>IF(A33="","",IF(ISNUMBER(C33),C33,B33))</f>
         <v/>
       </c>
-      <c r="E33" s="16" t="n"/>
+      <c r="E33" s="16" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="16" t="inlineStr"/>
@@ -2158,7 +2194,7 @@
         <f>IF(A34="","",IF(ISNUMBER(C34),C34,B34))</f>
         <v/>
       </c>
-      <c r="E34" s="16" t="n"/>
+      <c r="E34" s="16" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2239,7 +2275,7 @@
       </c>
       <c r="B5" s="16" t="inlineStr">
         <is>
-          <t>김디자이너</t>
+          <t>정수현(Gongdee)</t>
         </is>
       </c>
       <c r="C5" s="16" t="inlineStr">
@@ -2265,7 +2301,7 @@
       </c>
       <c r="B6" s="16" t="inlineStr">
         <is>
-          <t>박디자이너</t>
+          <t>문지선(Sun)</t>
         </is>
       </c>
       <c r="C6" s="16" t="inlineStr">
@@ -2291,7 +2327,7 @@
       </c>
       <c r="B7" s="16" t="inlineStr">
         <is>
-          <t>이디자이너</t>
+          <t>한수민(Stella)</t>
         </is>
       </c>
       <c r="C7" s="16" t="inlineStr">

</xml_diff>